<commit_message>
allows hydrogen prices to be affected by changes in production costs
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/BAEPAbCiPC/Bool Are Energy Prices Affected by Chng in Production Costs.xlsx
+++ b/InputData/ctrl-settings/BAEPAbCiPC/Bool Are Energy Prices Affected by Chng in Production Costs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\BAEPAbCiPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\BAEPAbCiPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEA0A00-D6A6-4D26-8247-961C9C80FF62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE87DAF9-09EA-470F-9ADE-533C67AF7202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1335" yWindow="5955" windowWidth="19185" windowHeight="11265" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -469,14 +469,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,22 +484,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -516,18 +516,18 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" width="33.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -535,7 +535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -559,7 +559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -567,7 +567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -575,7 +575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -583,7 +583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -591,7 +591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -599,7 +599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -607,7 +607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -615,7 +615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -623,7 +623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -631,7 +631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -639,7 +639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -647,7 +647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -655,7 +655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -663,7 +663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -671,7 +671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>25</v>
       </c>
@@ -687,12 +687,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BAEPAbCiPC set hydrogen to 0
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/BAEPAbCiPC/Bool Are Energy Prices Affected by Chng in Production Costs.xlsx
+++ b/InputData/ctrl-settings/BAEPAbCiPC/Bool Are Energy Prices Affected by Chng in Production Costs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\BAEPAbCiPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\ctrl-settings\BAEPAbCiPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE87DAF9-09EA-470F-9ADE-533C67AF7202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF07184-BD60-4A62-8D9E-0F1013B3348F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1335" yWindow="5955" windowWidth="19185" windowHeight="11265" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -469,14 +469,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,22 +484,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -516,18 +516,18 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.81640625" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -535,7 +535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -543,7 +543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -551,7 +551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>
@@ -559,7 +559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -567,7 +567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -575,7 +575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -583,7 +583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -591,7 +591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -599,7 +599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -607,7 +607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -615,7 +615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -623,7 +623,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -631,7 +631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -639,7 +639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -647,7 +647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -655,7 +655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -663,7 +663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -671,7 +671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>25</v>
       </c>
@@ -687,12 +687,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>